<commit_message>
Update Kimi K3's evaluation results on Protocol III
</commit_message>
<xml_diff>
--- a/docs/static/data/webretriever_results.xlsx
+++ b/docs/static/data/webretriever_results.xlsx
@@ -1,8 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Desktop\OS-World.github.io-main\static\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
     <workbookView windowWidth="23040" windowHeight="9180"/>
   </bookViews>
@@ -27,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="44">
   <si>
     <t>Agent</t>
   </si>
@@ -144,6 +149,21 @@
   </si>
   <si>
     <t>Anthropic, 25</t>
+  </si>
+  <si>
+    <t>Kimi Agent</t>
+  </si>
+  <si>
+    <t>Kimi K3</t>
+  </si>
+  <si>
+    <t>Moonshot AI</t>
+  </si>
+  <si>
+    <t>https://www.kimi.com/blog/kimi-k3</t>
+  </si>
+  <si>
+    <t>Kimi Team, 26</t>
   </si>
 </sst>
 </file>
@@ -1639,7 +1659,7 @@
       <c r="N7" s="7"/>
       <c r="O7" s="7"/>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" ht="13.95" spans="1:15">
       <c r="A8" s="7" t="s">
         <v>34</v>
       </c>
@@ -1679,17 +1699,31 @@
       <c r="O8" s="7"/>
     </row>
     <row r="9" ht="21" customHeight="1" spans="1:15">
-      <c r="A9" s="7"/>
-      <c r="B9" s="13"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13"/>
+      <c r="A9" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="F9" s="13">
+        <v>46226</v>
+      </c>
+      <c r="G9" s="7"/>
       <c r="H9" s="7"/>
       <c r="I9" s="7"/>
       <c r="J9" s="7"/>
-      <c r="K9" s="7"/>
+      <c r="K9" s="7">
+        <v>28</v>
+      </c>
       <c r="L9" s="7"/>
       <c r="M9" s="7"/>
       <c r="N9" s="7"/>
@@ -16682,6 +16716,7 @@
     <hyperlink ref="D4" r:id="rId4" display="https://arxiv.org/abs/2407.13032" tooltip="https://arxiv.org/abs/2407.13032"/>
     <hyperlink ref="D8" r:id="rId5" display="https://www.anthropic.com/news/claude-sonnet-4-5" tooltip="https://www.anthropic.com/news/claude-sonnet-4-5"/>
     <hyperlink ref="D7" r:id="rId6" display="https://arxiv.org/abs/2507.06261"/>
+    <hyperlink ref="D9" r:id="rId7" display="https://www.kimi.com/blog/kimi-k3"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
Update evaluation results on Protocol III
</commit_message>
<xml_diff>
--- a/docs/static/data/webretriever_results.xlsx
+++ b/docs/static/data/webretriever_results.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="47">
   <si>
     <t>Agent</t>
   </si>
@@ -164,6 +164,15 @@
   </si>
   <si>
     <t>Kimi Team, 26</t>
+  </si>
+  <si>
+    <t>claude-4-8-opus</t>
+  </si>
+  <si>
+    <t>https://www.anthropic.com/news/claude-opus-4-8</t>
+  </si>
+  <si>
+    <t>Anthropic, 26</t>
   </si>
 </sst>
 </file>
@@ -1730,17 +1739,31 @@
       <c r="O9" s="7"/>
     </row>
     <row r="10" ht="13.95" spans="1:15">
-      <c r="A10" s="7"/>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
+      <c r="A10" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="F10" s="13">
+        <v>46227</v>
+      </c>
       <c r="G10" s="7"/>
       <c r="H10" s="7"/>
       <c r="I10" s="7"/>
       <c r="J10" s="7"/>
-      <c r="K10" s="7"/>
+      <c r="K10" s="7">
+        <v>47</v>
+      </c>
       <c r="L10" s="7"/>
       <c r="M10" s="7"/>
       <c r="N10" s="7"/>
@@ -1750,7 +1773,7 @@
       <c r="A11" s="7"/>
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
+      <c r="D11" s="12"/>
       <c r="E11" s="13"/>
       <c r="F11" s="13"/>
       <c r="G11" s="14"/>
@@ -16717,6 +16740,7 @@
     <hyperlink ref="D8" r:id="rId5" display="https://www.anthropic.com/news/claude-sonnet-4-5" tooltip="https://www.anthropic.com/news/claude-sonnet-4-5"/>
     <hyperlink ref="D7" r:id="rId6" display="https://arxiv.org/abs/2507.06261"/>
     <hyperlink ref="D9" r:id="rId7" display="https://www.kimi.com/blog/kimi-k3"/>
+    <hyperlink ref="D10" r:id="rId8" display="https://www.anthropic.com/news/claude-opus-4-8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>